<commit_message>
Remove venv from repository
</commit_message>
<xml_diff>
--- a/Project_002 - Create port configuration based on Excel File/portmapping.xlsx
+++ b/Project_002 - Create port configuration based on Excel File/portmapping.xlsx
@@ -46,19 +46,19 @@
     <t xml:space="preserve">g0/1</t>
   </si>
   <si>
-    <t xml:space="preserve">Device 1</t>
+    <t xml:space="preserve">test1</t>
   </si>
   <si>
     <t xml:space="preserve">g0/2</t>
   </si>
   <si>
-    <t xml:space="preserve">PC1</t>
+    <t xml:space="preserve">test2</t>
   </si>
   <si>
     <t xml:space="preserve">g0/3</t>
   </si>
   <si>
-    <t xml:space="preserve">Laptop10</t>
+    <t xml:space="preserve">teste3</t>
   </si>
   <si>
     <t xml:space="preserve">g0/4</t>
@@ -190,28 +190,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -407,207 +411,207 @@
   <dimension ref="A1:E29"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>21</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>50</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>51</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>40</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>160</v>
       </c>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5" t="s">
+      <c r="C8" s="6"/>
+      <c r="D8" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>130</v>
       </c>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5" t="s">
+      <c r="C9" s="6"/>
+      <c r="D9" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5" t="s">
+      <c r="C10" s="6"/>
+      <c r="D10" s="6" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5" t="s">
+      <c r="C11" s="6"/>
+      <c r="D11" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="s">
+      <c r="A12" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5" t="s">
+      <c r="C12" s="6"/>
+      <c r="D12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4"/>
+      <c r="A13" s="5"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4"/>
+      <c r="A14" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4"/>
+      <c r="A15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4"/>
+      <c r="A16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4"/>
+      <c r="A17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4"/>
+      <c r="A18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4"/>
+      <c r="A19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4"/>
+      <c r="A20" s="5"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4"/>
+      <c r="A21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4"/>
+      <c r="A22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4"/>
+      <c r="A23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4"/>
+      <c r="A24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4"/>
+      <c r="A25" s="5"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4"/>
+      <c r="A26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4"/>
+      <c r="A27" s="5"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4"/>
+      <c r="A28" s="5"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4"/>
+      <c r="A29" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>